<commit_message>
feat: add UI31 skill testing and stabilize battle lifecycle
</commit_message>
<xml_diff>
--- a/exports/level_configuration_current/当前关卡配置.xlsx
+++ b/exports/level_configuration_current/当前关卡配置.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>1e072221efbaf4a195545a01faec1ef93f5bb13bc87f19467876df819611eb9a</t>
+          <t>a9d9cd2925b4e9deab4c67eea04eb8f678c598cd63813f6d201941f97308b319</t>
         </is>
       </c>
     </row>
@@ -5927,7 +5927,7 @@
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr"/>
       <c r="T30" s="5" t="n">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="U30" s="5" t="inlineStr"/>
       <c r="V30" s="5" t="n">
@@ -10605,7 +10605,7 @@
       <c r="R70" s="5" t="inlineStr"/>
       <c r="S70" s="5" t="inlineStr"/>
       <c r="T70" s="5" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="U70" s="5" t="inlineStr"/>
       <c r="V70" s="5" t="n">
@@ -17471,7 +17471,7 @@
       <c r="R126" s="5" t="inlineStr"/>
       <c r="S126" s="5" t="inlineStr"/>
       <c r="T126" s="5" t="n">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="U126" s="5" t="inlineStr"/>
       <c r="V126" s="5" t="n">

</xml_diff>